<commit_message>
fix: build LinkedIn embed URLs from new post URLs
New LinkedIn exports use /posts/<slug>-<type>-<id>-<suffix> URLs. The
app used the last path segment as the embed ID, so LinkedIn returned
404 for these posts. Add getLinkedInEmbedUrl to get the URN from old
and new URL shapes, and use it in the top posts grid and the Peak
Performer card.

Add Vitest and tests for the helper. Change most demo URLs to the new
shape and keep one old URL, so that sample data tests both shapes.

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/site/public/demo-data/linkedin-demo.xlsx
+++ b/site/public/demo-data/linkedin-demo.xlsx
@@ -1143,157 +1143,157 @@
     <t/>
   </si>
   <si>
-    <t>https://www.linkedin.com/feed/update/urn:li:activity:7354518350980341760</t>
+    <t>https://www.linkedin.com/posts/shifra-williams_its-bonkers-that-the-most-effective-way-share-7435833322456436736-mUmk</t>
   </si>
   <si>
     <t>https://www.linkedin.com/feed/update/urn:li:activity:7366110943438589952</t>
   </si>
   <si>
-    <t>https://www.linkedin.com/feed/update/urn:li:activity:7359591750698471424</t>
-  </si>
-  <si>
-    <t>https://www.linkedin.com/feed/update/urn:li:activity:7308967160444342273</t>
-  </si>
-  <si>
-    <t>https://www.linkedin.com/feed/update/urn:li:activity:7369376285426425858</t>
-  </si>
-  <si>
-    <t>https://www.linkedin.com/feed/update/urn:li:activity:7369753714145906688</t>
-  </si>
-  <si>
-    <t>https://www.linkedin.com/feed/update/urn:li:activity:7279185671762718720</t>
-  </si>
-  <si>
-    <t>https://www.linkedin.com/feed/update/urn:li:activity:7275661708310810625</t>
-  </si>
-  <si>
-    <t>https://www.linkedin.com/feed/update/urn:li:activity:7351253040978378752</t>
-  </si>
-  <si>
-    <t>https://www.linkedin.com/feed/update/urn:li:activity:7306446546009575424</t>
-  </si>
-  <si>
-    <t>https://www.linkedin.com/feed/update/urn:li:activity:7389685083613339648</t>
-  </si>
-  <si>
-    <t>https://www.linkedin.com/feed/update/urn:li:activity:7332790149065445376</t>
-  </si>
-  <si>
-    <t>https://www.linkedin.com/feed/update/urn:li:activity:7311050646558760960</t>
-  </si>
-  <si>
-    <t>https://www.linkedin.com/feed/update/urn:li:activity:7344016674318106625</t>
-  </si>
-  <si>
-    <t>https://www.linkedin.com/feed/update/urn:li:activity:7355964071638147072</t>
-  </si>
-  <si>
-    <t>https://www.linkedin.com/feed/update/urn:li:activity:7308525598803480576</t>
-  </si>
-  <si>
-    <t>https://www.linkedin.com/feed/update/urn:li:activity:7295942675831095296</t>
-  </si>
-  <si>
-    <t>https://www.linkedin.com/feed/update/urn:li:activity:7340385179087081472</t>
-  </si>
-  <si>
-    <t>https://www.linkedin.com/feed/update/urn:li:activity:7376623992893239296</t>
-  </si>
-  <si>
-    <t>https://www.linkedin.com/feed/update/urn:li:activity:7360678945240850432</t>
-  </si>
-  <si>
-    <t>https://www.linkedin.com/feed/update/urn:li:activity:7341902678484037634</t>
-  </si>
-  <si>
-    <t>https://www.linkedin.com/feed/update/urn:li:activity:7361048826788413442</t>
-  </si>
-  <si>
-    <t>https://www.linkedin.com/feed/update/urn:li:activity:7366480888823439360</t>
-  </si>
-  <si>
-    <t>https://www.linkedin.com/feed/update/urn:li:activity:7354171041142718466</t>
-  </si>
-  <si>
-    <t>https://www.linkedin.com/feed/update/urn:li:activity:7365752407684726784</t>
-  </si>
-  <si>
-    <t>https://www.linkedin.com/feed/update/urn:li:activity:7334232128420827137</t>
-  </si>
-  <si>
-    <t>https://www.linkedin.com/feed/update/urn:li:activity:7311452043422957571</t>
-  </si>
-  <si>
-    <t>https://www.linkedin.com/feed/update/urn:li:activity:7322639488566890497</t>
-  </si>
-  <si>
-    <t>https://www.linkedin.com/feed/update/urn:li:activity:7364680261269090304</t>
-  </si>
-  <si>
-    <t>https://www.linkedin.com/feed/update/urn:li:activity:7384600277535969280</t>
-  </si>
-  <si>
-    <t>https://www.linkedin.com/feed/update/urn:li:activity:7310451876947189760</t>
-  </si>
-  <si>
-    <t>https://www.linkedin.com/feed/update/urn:li:activity:7386400978440179712</t>
-  </si>
-  <si>
-    <t>https://www.linkedin.com/feed/update/urn:li:activity:7375918487682297856</t>
-  </si>
-  <si>
-    <t>https://www.linkedin.com/feed/update/urn:li:activity:7394732042997116928</t>
-  </si>
-  <si>
-    <t>https://www.linkedin.com/feed/update/urn:li:activity:7350532051038572544</t>
-  </si>
-  <si>
-    <t>https://www.linkedin.com/feed/update/urn:li:activity:7372275372643749888</t>
-  </si>
-  <si>
-    <t>https://www.linkedin.com/feed/update/urn:li:activity:7379164450970415105</t>
-  </si>
-  <si>
-    <t>https://www.linkedin.com/feed/update/urn:li:activity:7374457289954496512</t>
-  </si>
-  <si>
-    <t>https://www.linkedin.com/feed/update/urn:li:activity:7318664580442775553</t>
-  </si>
-  <si>
-    <t>https://www.linkedin.com/feed/update/urn:li:activity:7318302193428680711</t>
-  </si>
-  <si>
-    <t>https://www.linkedin.com/feed/update/urn:li:activity:7381712556714921984</t>
-  </si>
-  <si>
-    <t>https://www.linkedin.com/feed/update/urn:li:activity:7348697462636744704</t>
-  </si>
-  <si>
-    <t>https://www.linkedin.com/feed/update/urn:li:activity:7358206776430796801</t>
-  </si>
-  <si>
-    <t>https://www.linkedin.com/feed/update/urn:li:activity:7349437390320484353</t>
-  </si>
-  <si>
-    <t>https://www.linkedin.com/feed/update/urn:li:activity:7392214274271563777</t>
-  </si>
-  <si>
-    <t>https://www.linkedin.com/feed/update/urn:li:activity:7396517542548381696</t>
-  </si>
-  <si>
-    <t>https://www.linkedin.com/feed/update/urn:li:activity:7388937604433600512</t>
-  </si>
-  <si>
-    <t>https://www.linkedin.com/feed/update/urn:li:activity:7336028985576841216</t>
-  </si>
-  <si>
-    <t>https://www.linkedin.com/feed/update/urn:li:activity:7315033150403874816</t>
-  </si>
-  <si>
-    <t>https://www.linkedin.com/feed/update/urn:li:activity:7343284287707750403</t>
-  </si>
-  <si>
-    <t>https://www.linkedin.com/feed/update/urn:li:activity:7310001438842122240</t>
+    <t>https://www.linkedin.com/posts/shifra-williams_hosting-3-speakers-with-basically-identical-ugcPost-7470288868446162944-J0Pq</t>
+  </si>
+  <si>
+    <t>https://www.linkedin.com/posts/shifra-williams_%F0%9D%90%8C%F0%9D%90%A8%F0%9D%90%AC%F0%9D%90%AD-%F0%9D%90%A9%F0%9D%90%9E%F0%9D%90%A8%F0%9D%90%A9%F0%9D%90%A5%F0%9D%90%9E-%F0%9D%90%A8%F0%9D%90%A7-%F0%9D%90%8B%F0%9D%90%A2%F0%9D%90%A7%F0%9D%90%A4%F0%9D%90%9E%F0%9D%90%9D%F0%9D%90%88-share-7387636325484769280-YVpH</t>
+  </si>
+  <si>
+    <t>https://www.linkedin.com/posts/shifra-williams_a-recruiter-slid-into-my-dms-recently-with-share-7435847472301817856-J8WT</t>
+  </si>
+  <si>
+    <t>https://www.linkedin.com/posts/shifra-williams_wrappedforlinkedin-2025recap-ugcPost-7406869077442408448-tUDn</t>
+  </si>
+  <si>
+    <t>https://www.linkedin.com/posts/shifra-williams_shivampatelresume-ugcPost-7416305335683956736-qq39</t>
+  </si>
+  <si>
+    <t>https://www.linkedin.com/posts/shifra-williams_wrapped-ugcPost-7406875180880502784-A3se</t>
+  </si>
+  <si>
+    <t>https://www.linkedin.com/posts/shifra-williams_dataengineering-python-pandas-share-7432338576400449537-jiD1</t>
+  </si>
+  <si>
+    <t>https://www.linkedin.com/posts/shifra-williams_big-news-i-recently-joined-render-the-cloud-share-7405420483900301312-148b</t>
+  </si>
+  <si>
+    <t>https://www.linkedin.com/posts/shifra-williams_cant-believe-im-working-with-the-one-and-share-7448863044811644929-Q4u4</t>
+  </si>
+  <si>
+    <t>https://www.linkedin.com/posts/shifra-williams_hazal-mestci-and-i-just-wrapped-up-the-mcp-ugcPost-7445938294460370944-pifd</t>
+  </si>
+  <si>
+    <t>https://www.linkedin.com/posts/shifra-williams_apparently-my-new-google-gemini-generated-share-7444532479534821376-C80_</t>
+  </si>
+  <si>
+    <t>https://www.linkedin.com/posts/shifra-williams_loved-meeting-chang-she-one-of-the-original-ugcPost-7437659850848960512-K29L</t>
+  </si>
+  <si>
+    <t>https://www.linkedin.com/posts/shifra-williams_ive-been-staring-at-my-linkedin-drafts-for-share-7405417305481916416-MOqA</t>
+  </si>
+  <si>
+    <t>https://www.linkedin.com/posts/shifra-williams_osidalkurdresumepdf-ugcPost-7415541853950971904-yR0D</t>
+  </si>
+  <si>
+    <t>https://www.linkedin.com/posts/shifra-williams_she-ships-reminded-me-why-community-events-ugcPost-7435850358188343296-cghX</t>
+  </si>
+  <si>
+    <t>https://www.linkedin.com/posts/shifra-williams_thought-anthropic-claude-was-working-on-something-share-7455002587067682817-O-wg</t>
+  </si>
+  <si>
+    <t>https://www.linkedin.com/posts/shifra-williams_last-week-i-got-to-demo-my-rag-pipeline-at-ugcPost-7448868000985792512--38b</t>
+  </si>
+  <si>
+    <t>https://www.linkedin.com/posts/shifra-williams_github-brand-ugcPost-7385845292233048064-2nxT</t>
+  </si>
+  <si>
+    <t>https://www.linkedin.com/posts/shifra-williams_agenticai-hackathon-share-7485528159346622464-sQj-</t>
+  </si>
+  <si>
+    <t>https://www.linkedin.com/posts/shifra-williams_pride-luma-share-7474294718445604865-RkX0</t>
+  </si>
+  <si>
+    <t>https://www.linkedin.com/posts/shifra-williams_london-im-coming-for-you-ill-be-representing-share-7443394147018780673-QAAW</t>
+  </si>
+  <si>
+    <t>https://www.linkedin.com/posts/shifra-williams_datascience-statistics-saturdata-share-7432338052053860354-NfuM</t>
+  </si>
+  <si>
+    <t>https://www.linkedin.com/posts/shifra-williams_i-just-won-document360s-global-writers-share-7415555050543980544-hjFw</t>
+  </si>
+  <si>
+    <t>https://www.linkedin.com/posts/shifra-williams_just-because-i-havent-posted-about-it-yet-ugcPost-7453940757498859520--1fx</t>
+  </si>
+  <si>
+    <t>https://www.linkedin.com/posts/shifra-williams_shifrasolutionscom-domain-for-sale-share-7435850946204790784-TPLY</t>
+  </si>
+  <si>
+    <t>https://www.linkedin.com/posts/shifra-williams_ive-been-in-tech-long-enough-to-know-that-share-7421629614545895424-eFaH</t>
+  </si>
+  <si>
+    <t>https://www.linkedin.com/posts/shifra-williams_got-to-visit-the-amazon-web-services-aws-share-7423543316950192128-iJ38</t>
+  </si>
+  <si>
+    <t>https://www.linkedin.com/posts/shifra-williams_motherduck-ugcPost-7379973989634584576-KsqY</t>
+  </si>
+  <si>
+    <t>https://www.linkedin.com/posts/shifra-williams_im-thrilled-to-announce-that-ill-be-speaking-share-7382851133901312000-fMcA</t>
+  </si>
+  <si>
+    <t>https://www.linkedin.com/posts/shifra-williams_why-render-is-the-fastest-path-to-production-share-7453936563698176000-sakG</t>
+  </si>
+  <si>
+    <t>https://www.linkedin.com/posts/shifra-williams_datascience-aifluency-aisafety-share-7432338761172254720-862-</t>
+  </si>
+  <si>
+    <t>https://www.linkedin.com/posts/shifra-williams_getting-an-unconditional-offer-to-a-masters-ugcPost-7452026808964771840-pO0u</t>
+  </si>
+  <si>
+    <t>https://www.linkedin.com/posts/shifra-williams_last-week-i-had-the-chance-to-attend-a-motherduck-share-7382853310917165056-gyOW</t>
+  </si>
+  <si>
+    <t>https://www.linkedin.com/posts/shifra-williams_dim-sum-sushi-boba-and-a-photo-booth-ugcPost-7451898030787776513-JT7r</t>
+  </si>
+  <si>
+    <t>https://www.linkedin.com/posts/shifra-williams_just-finished-martin-kleppmanns-designing-ugcPost-7390914248807251968-4Idi</t>
+  </si>
+  <si>
+    <t>https://www.linkedin.com/posts/shifra-williams_jos%C3%A9-siles-is-always-top-tier-share-7446593341468717056-J5V4</t>
+  </si>
+  <si>
+    <t>https://www.linkedin.com/posts/shifra-williams_better-late-than-never-my-london-trip-gave-ugcPost-7453934591343771648-toO_</t>
+  </si>
+  <si>
+    <t>https://www.linkedin.com/posts/shifra-williams_i-just-dropped-my-first-video-tutorial-with-share-7419847633147547652-ZmbG</t>
+  </si>
+  <si>
+    <t>https://www.linkedin.com/posts/shifra-williams_lsmtreesbtrees-ugcPost-7387630390422962176-RGPk</t>
+  </si>
+  <si>
+    <t>https://www.linkedin.com/posts/shifra-williams_datascience-dataengineering-python-share-7398946669205143552-ECL8</t>
+  </si>
+  <si>
+    <t>https://www.linkedin.com/posts/shifra-williams_%F0%9D%90%93%F0%9D%90%A1%F0%9D%90%A2%F0%9D%90%AC-%F0%9D%90%A2%F0%9D%90%AC-%F0%9D%90%A1%F0%9D%90%A8%F0%9D%90%B0-%F0%9D%90%88-%F0%9D%90%B0%F0%9D%90%9E%F0%9D%90%A7%F0%9D%90%AD-%F0%9D%90%9F%F0%9D%90%AB%F0%9D%90%A8%F0%9D%90%A6-share-7412631213737439232-p8Cc</t>
+  </si>
+  <si>
+    <t>https://www.linkedin.com/posts/shifra-williams_saturdata-interviews-share-7419845929647915009-Ktz3</t>
+  </si>
+  <si>
+    <t>https://www.linkedin.com/posts/shifra-williams_scd-ugcPost-7382849839383859200-dttY</t>
+  </si>
+  <si>
+    <t>https://www.linkedin.com/posts/shifra-williams_so-excited-for-developers-to-see-this-share-7503867900148199425-FxMI</t>
+  </si>
+  <si>
+    <t>https://www.linkedin.com/posts/shifra-williams_redefiningcareers-ugcPost-7470834209478336512-DvPE</t>
+  </si>
+  <si>
+    <t>https://www.linkedin.com/posts/shifra-williams_happy-pride-month-to-all-my-kings-queens-share-7470293529810919424-SxyQ</t>
+  </si>
+  <si>
+    <t>https://www.linkedin.com/posts/shifra-williams_%F0%9D%90%88-%F0%9D%90%A9%F0%9D%90%AB%F0%9D%90%A8%F0%9D%90%A6%F0%9D%90%A8%F0%9D%90%AD%F0%9D%90%9E%F0%9D%90%9D-%F0%9D%90%82%F0%9D%90%A5%F0%9D%90%9A%F0%9D%90%AE%F0%9D%90%9D%F0%9D%90%9E-%F0%9D%90%AD%F0%9D%90%A8-share-7392711214080077825-u08d</t>
+  </si>
+  <si>
+    <t>https://www.linkedin.com/posts/shifra-williams_sqlwinning-ugcPost-7385842965824352256-4XoZ</t>
+  </si>
+  <si>
+    <t>https://www.linkedin.com/posts/shifra-williams_once-upon-a-time-i-sat-down-at-a-caltrain-share-7412631762025033729-JmrG</t>
   </si>
   <si>
     <t>https://www.linkedin.com/feed/update/urn:li:activity:7381342582137651200</t>

</xml_diff>